<commit_message>
Update workshop data and methods
</commit_message>
<xml_diff>
--- a/data/2B_descent.xlsx
+++ b/data/2B_descent.xlsx
@@ -1154,7 +1154,7 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>What the data says: the residual table (24 corridors after shipping, timing and the hub)</t>
+          <t>What the data says: the table of what is left unexplained (24 corridors after shipping, timing and the hub)</t>
         </is>
       </c>
       <c r="B6" s="12" t="n"/>
@@ -1182,7 +1182,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>A bin per corridor, and a first check for every investigate (required)</t>
+          <t>A bin for each corridor, and a first check for each one marked investigate (required)</t>
         </is>
       </c>
       <c r="B8" s="2" t="n"/>
@@ -1554,7 +1554,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>The corridor to descend into</t>
+          <t>The corridor to look into</t>
         </is>
       </c>
       <c r="B34" s="12" t="n"/>
@@ -1610,7 +1610,7 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>What a wrong bin costs, in one line</t>
+          <t>What a wrong bin costs (one sentence)</t>
         </is>
       </c>
       <c r="B38" s="12" t="n"/>
@@ -1796,7 +1796,7 @@
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>The one never to open</t>
+          <t>The importer never to open</t>
         </is>
       </c>
       <c r="B51" s="12" t="n"/>
@@ -2030,7 +2030,7 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>That the range is never a value, in one line</t>
+          <t>One sentence saying the range is never a value</t>
         </is>
       </c>
       <c r="B68" s="12" t="n"/>
@@ -19825,7 +19825,7 @@
       </c>
       <c r="B7" s="37" t="inlineStr">
         <is>
-          <t>The lines we compare a line with: same goods, same origin, last 12 months, widened when too few</t>
+          <t>The lines we compare a line with: same goods, same origin, last 12 months, widened when there are too few</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -19995,7 +19995,7 @@
       </c>
       <c r="B17" s="37" t="inlineStr">
         <is>
-          <t>What home recorded against what the partner says it shipped</t>
+          <t>What the home country recorded against what the partner says it shipped</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -20012,7 +20012,7 @@
       </c>
       <c r="B18" s="37" t="inlineStr">
         <is>
-          <t>Why home imports (CIF) sit above partner exports (FOB)</t>
+          <t>Why the home country's imports (CIF) sit above the partner's exports (FOB)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="B26" s="37" t="inlineStr">
         <is>
-          <t>The list of every table and column with its meaning, its source system and its refresh, and for every computed number the inputs and the window it came from</t>
+          <t>The list of every table and column with its meaning, source system and refresh; and, for every computed number, the inputs and the time window it came from</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data-v12: Breakout 4B v2 four lists (ADD-L), recipe text before the gate (ADD-I I.12)
</commit_message>
<xml_diff>
--- a/data/2B_descent.xlsx
+++ b/data/2B_descent.xlsx
@@ -72306,12 +72306,12 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Bucket</t>
+          <t>The four lists</t>
         </is>
       </c>
       <c r="B23" s="37" t="inlineStr">
         <is>
-          <t>The group an importer falls in: unregistered, not filing, under-reporting, consistent</t>
+          <t>Where an importer lands when it fails one of four questions asked in order: not known to tax, not filing, import not in its books, sells below what it imports</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">

</xml_diff>